<commit_message>
remove item Síndrome Gripal da navbar
</commit_message>
<xml_diff>
--- a/tabelas/srag_15rs_2026.xlsx
+++ b/tabelas/srag_15rs_2026.xlsx
@@ -774,7 +774,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -899,10 +899,10 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>411640</v>
+        <v>411690</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -911,18 +911,18 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NOSSA SENHORA DAS GRACAS</t>
+          <t>NOVA ESPERANCA</t>
         </is>
       </c>
       <c r="G4">
-        <v>3669</v>
+        <v>27142</v>
       </c>
       <c r="H4">
-        <v>54.5</v>
+        <v>55.3</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -933,7 +933,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>412530</v>
+        <v>411640</v>
       </c>
       <c r="B5">
         <v>2</v>
@@ -945,18 +945,18 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SAO JORGE DO IVAI</t>
+          <t>NOSSA SENHORA DAS GRACAS</t>
         </is>
       </c>
       <c r="G5">
-        <v>5170</v>
+        <v>3669</v>
       </c>
       <c r="H5">
-        <v>38.7</v>
+        <v>54.5</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -967,10 +967,10 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>411690</v>
+        <v>411090</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -983,14 +983,14 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>NOVA ESPERANCA</t>
+          <t>ITAGUAJE</t>
         </is>
       </c>
       <c r="G6">
-        <v>27142</v>
+        <v>4530</v>
       </c>
       <c r="H6">
-        <v>36.8</v>
+        <v>44.2</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1001,10 +1001,10 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>411740</v>
+        <v>412530</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1017,14 +1017,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>OURIZONA</t>
+          <t>SAO JORGE DO IVAI</t>
         </is>
       </c>
       <c r="G7">
-        <v>3193</v>
+        <v>5170</v>
       </c>
       <c r="H7">
-        <v>31.3</v>
+        <v>38.7</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1038,16 +1038,16 @@
         <v>411520</v>
       </c>
       <c r="B8">
-        <v>122</v>
+        <v>155</v>
       </c>
       <c r="C8">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D8">
         <v>2</v>
       </c>
       <c r="E8">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1058,21 +1058,21 @@
         <v>429660</v>
       </c>
       <c r="H8">
-        <v>28.4</v>
+        <v>36.1</v>
       </c>
       <c r="I8">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="J8">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>410220</v>
+        <v>411110</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1085,14 +1085,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ATALAIA</t>
+          <t>ITAMBE</t>
         </is>
       </c>
       <c r="G9">
-        <v>4046</v>
+        <v>6228</v>
       </c>
       <c r="H9">
-        <v>24.7</v>
+        <v>32.1</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>411630</v>
+        <v>411740</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1115,18 +1115,18 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MUNHOZ DE MELO</t>
+          <t>OURIZONA</t>
         </is>
       </c>
       <c r="G10">
-        <v>4057</v>
+        <v>3193</v>
       </c>
       <c r="H10">
-        <v>24.6</v>
+        <v>31.3</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1137,78 +1137,78 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>410590</v>
+        <v>412625</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>COLORADO</t>
+          <t>SARANDI</t>
         </is>
       </c>
       <c r="G11">
-        <v>23313</v>
+        <v>128106</v>
       </c>
       <c r="H11">
-        <v>21.4</v>
+        <v>28.9</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>411810</v>
+        <v>411480</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PARANACITY</t>
+          <t>MARIALVA</t>
         </is>
       </c>
       <c r="G12">
-        <v>9549</v>
+        <v>44749</v>
       </c>
       <c r="H12">
-        <v>20.9</v>
+        <v>26.8</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="J12">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>410780</v>
+        <v>410590</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1217,18 +1217,18 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FLORAI</t>
+          <t>COLORADO</t>
         </is>
       </c>
       <c r="G13">
-        <v>4805</v>
+        <v>23313</v>
       </c>
       <c r="H13">
-        <v>20.8</v>
+        <v>25.7</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1239,10 +1239,10 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>411410</v>
+        <v>410220</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1251,18 +1251,18 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MANDAGUACU</t>
+          <t>ATALAIA</t>
         </is>
       </c>
       <c r="G14">
-        <v>34521</v>
+        <v>4046</v>
       </c>
       <c r="H14">
-        <v>20.3</v>
+        <v>24.7</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1273,64 +1273,64 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>412625</v>
+        <v>411630</v>
       </c>
       <c r="B15">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E15">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SARANDI</t>
+          <t>MUNHOZ DE MELO</t>
         </is>
       </c>
       <c r="G15">
-        <v>128106</v>
+        <v>4057</v>
       </c>
       <c r="H15">
-        <v>20.3</v>
+        <v>24.6</v>
       </c>
       <c r="I15">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>3.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>411480</v>
+        <v>411410</v>
       </c>
       <c r="B16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>MARIALVA</t>
+          <t>MANDAGUACU</t>
         </is>
       </c>
       <c r="G16">
-        <v>44749</v>
+        <v>34521</v>
       </c>
       <c r="H16">
-        <v>20.1</v>
+        <v>23.2</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -1341,64 +1341,64 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>411750</v>
+        <v>411360</v>
       </c>
       <c r="B17">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PAICANDU</t>
+          <t>LOBATO</t>
         </is>
       </c>
       <c r="G17">
-        <v>48695</v>
+        <v>4707</v>
       </c>
       <c r="H17">
-        <v>16.4</v>
+        <v>21.2</v>
       </c>
       <c r="I17">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="J17">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>411110</v>
+        <v>411810</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ITAMBE</t>
+          <t>PARANACITY</t>
         </is>
       </c>
       <c r="G18">
-        <v>6228</v>
+        <v>9549</v>
       </c>
       <c r="H18">
-        <v>16.1</v>
+        <v>20.9</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -1409,7 +1409,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>410730</v>
+        <v>410780</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1425,14 +1425,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>DOUTOR CAMARGO</t>
+          <t>FLORAI</t>
         </is>
       </c>
       <c r="G19">
-        <v>6517</v>
+        <v>4805</v>
       </c>
       <c r="H19">
-        <v>15.3</v>
+        <v>20.8</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -1443,30 +1443,30 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>411420</v>
+        <v>411000</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>MANDAGUARI</t>
+          <t>IGUARACU</t>
         </is>
       </c>
       <c r="G20">
-        <v>38313</v>
+        <v>5693</v>
       </c>
       <c r="H20">
-        <v>7.8</v>
+        <v>17.6</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1477,35 +1477,137 @@
     </row>
     <row r="21">
       <c r="A21">
+        <v>411750</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PAICANDU</t>
+        </is>
+      </c>
+      <c r="G21">
+        <v>48695</v>
+      </c>
+      <c r="H21">
+        <v>16.4</v>
+      </c>
+      <c r="I21">
+        <v>2.1</v>
+      </c>
+      <c r="J21">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>410730</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>DOUTOR CAMARGO</t>
+        </is>
+      </c>
+      <c r="G22">
+        <v>6517</v>
+      </c>
+      <c r="H22">
+        <v>15.3</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>411420</v>
+      </c>
+      <c r="B23">
+        <v>4</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>MANDAGUARI</t>
+        </is>
+      </c>
+      <c r="G23">
+        <v>38313</v>
+      </c>
+      <c r="H23">
+        <v>10.4</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
         <v>410210</v>
       </c>
-      <c r="B21">
+      <c r="B24">
         <v>2</v>
       </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>ASTORGA</t>
         </is>
       </c>
-      <c r="G21">
+      <c r="G24">
         <v>26203</v>
       </c>
-      <c r="H21">
+      <c r="H24">
         <v>7.6</v>
       </c>
-      <c r="I21">
-        <v>0</v>
-      </c>
-      <c r="J21">
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
         <v>0</v>
       </c>
     </row>
@@ -1516,7 +1618,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1553,13 +1655,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1568,55 +1670,55 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PARQUE HORTENCIA</t>
+          <t>VILA MORANGUEIRA</t>
         </is>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VILA MORANGUEIRA</t>
+          <t>PARQUE HORTENCIA</t>
         </is>
       </c>
       <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
         <v>4</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
       <c r="E4">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALVORADA</t>
+          <t>JARDIM DIAMANTE</t>
         </is>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1625,17 +1727,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL REQUIAO</t>
+          <t>VILA MARUMBY</t>
         </is>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1644,17 +1746,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JARDIM TROPICAL</t>
+          <t>ZONA 07</t>
         </is>
       </c>
       <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
         <v>3</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1663,7 +1765,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PARQUE DAS LARANJEIRAS</t>
+          <t>ALVORADA</t>
         </is>
       </c>
       <c r="B8">
@@ -1682,45 +1784,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZONA 01</t>
+          <t>CONJUNTO HABITACIONAL INOCENTE</t>
         </is>
       </c>
       <c r="B9">
         <v>3</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ZONA 04</t>
+          <t>CONJUNTO HABITACIONAL REQUIAO</t>
         </is>
       </c>
       <c r="B10">
         <v>3</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>33.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ZONA 07</t>
+          <t>DISTRITO DE IGUATEMI IGUATEMI</t>
         </is>
       </c>
       <c r="B11">
@@ -1730,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -1739,17 +1841,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AEROPORTO</t>
+          <t>JARDIM SAO SILVESTRE</t>
         </is>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1758,30 +1860,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL INOCENTE</t>
+          <t>JARDIM TROPICAL</t>
         </is>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL SANENGE</t>
+          <t>PARQUE DAS LARANJEIRAS</t>
         </is>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1796,17 +1898,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CONJUNTO RESIDENCIAL RODOLPHO</t>
+          <t>ZONA 01</t>
         </is>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1815,26 +1917,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DISTRITO DE IGUATEMI IGUATEMI</t>
+          <t>ZONA 04</t>
         </is>
       </c>
       <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
         <v>2</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
       <c r="E16">
-        <v>0</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GREVILEAS</t>
+          <t>AEROPORTO</t>
         </is>
       </c>
       <c r="B17">
@@ -1844,7 +1946,7 @@
         <v>0</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1853,7 +1955,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>JARDIM DIAMANTE</t>
+          <t>CONJUNTO HABITACIONAL JOAO DE</t>
         </is>
       </c>
       <c r="B18">
@@ -1863,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1872,7 +1974,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JARDIM IPANEMA</t>
+          <t>CONJUNTO HABITACIONAL SANENGE</t>
         </is>
       </c>
       <c r="B19">
@@ -1891,7 +1993,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>JARDIM ITAIPU</t>
+          <t>CONJUNTO RESIDENCIAL RODOLPHO</t>
         </is>
       </c>
       <c r="B20">
@@ -1901,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -1910,7 +2012,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>JARDIM MONTE CARLO</t>
+          <t>GREVILEAS</t>
         </is>
       </c>
       <c r="B21">
@@ -1920,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1929,7 +2031,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>JARDIM PARAISO</t>
+          <t>JARDIM ITAIPU</t>
         </is>
       </c>
       <c r="B22">
@@ -1939,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1948,7 +2050,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>JARDIM SAO SILVESTRE</t>
+          <t>JARDIM MONTE CARLO</t>
         </is>
       </c>
       <c r="B23">
@@ -1958,7 +2060,7 @@
         <v>0</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -1967,112 +2069,112 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LOTEAMENTO SUMARE</t>
+          <t>JARDIM OASIS</t>
         </is>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PARQUE DAS GREVILEAS 3A PARTE</t>
+          <t>JARDIM OLIMPICO</t>
         </is>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VILA VARDELINA</t>
+          <t>JARDIM PARAISO</t>
         </is>
       </c>
       <c r="B26">
         <v>2</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ALTO DAS GREVILEAS</t>
+          <t>LOTEAMENTO SUMARE</t>
         </is>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ARMAZEM</t>
+          <t>PARQUE DAS GREVILEAS 3A PARTE</t>
         </is>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BOM JARDIM</t>
+          <t>PARQUE TARUMA</t>
         </is>
       </c>
       <c r="B29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -2081,17 +2183,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CHACARA PAULISTA</t>
+          <t>VILA ESPERANCA</t>
         </is>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -2100,11 +2202,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CIDADE UNIVERSITARIA</t>
+          <t>VILA SANTO ANTONIO</t>
         </is>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -2119,11 +2221,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL HERMANN</t>
+          <t>VILA VARDELINA</t>
         </is>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -2132,13 +2234,13 @@
         <v>1</v>
       </c>
       <c r="E32">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL JOAO DE</t>
+          <t>ALTO DAS GREVILEAS</t>
         </is>
       </c>
       <c r="B33">
@@ -2148,7 +2250,7 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -2157,7 +2259,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CONJUNTO HABITACIONAL KARINA</t>
+          <t>ARMAZEM</t>
         </is>
       </c>
       <c r="B34">
@@ -2176,7 +2278,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CONJUNTO JOAO DE BARRO CHAMPAG</t>
+          <t>BELA VISTA</t>
         </is>
       </c>
       <c r="B35">
@@ -2195,7 +2297,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CONJUNTO JOAO DE BARRO ITAPARI</t>
+          <t>BOM JARDIM</t>
         </is>
       </c>
       <c r="B36">
@@ -2205,7 +2307,7 @@
         <v>0</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2214,7 +2316,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CONJUNTO RESIDENCIAL CIDADE AL</t>
+          <t>CHACARA PAULISTA</t>
         </is>
       </c>
       <c r="B37">
@@ -2224,7 +2326,7 @@
         <v>0</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -2233,45 +2335,45 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>EBENEZER</t>
+          <t>CIDADE UNIVERSITARIA</t>
         </is>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IBIRAPUERA</t>
+          <t>CONJUNTO HABITACIONAL HERMANN</t>
         </is>
       </c>
       <c r="B39">
         <v>1</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IGUATEMI</t>
+          <t>CONJUNTO HABITACIONAL KARINA</t>
         </is>
       </c>
       <c r="B40">
@@ -2281,7 +2383,7 @@
         <v>0</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2290,7 +2392,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>JARDIM ALVORADA III</t>
+          <t>CONJUNTO JOAO DE BARRO CHAMPAG</t>
         </is>
       </c>
       <c r="B41">
@@ -2309,7 +2411,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>JARDIM BELA VISTA</t>
+          <t>CONJUNTO JOAO DE BARRO ITAPARI</t>
         </is>
       </c>
       <c r="B42">
@@ -2328,7 +2430,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>JARDIM BERTIOGA</t>
+          <t>CONJUNTO RESIDENCIAL CIDADE AL</t>
         </is>
       </c>
       <c r="B43">
@@ -2347,26 +2449,26 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>JARDIM DIAS I</t>
+          <t>CONJUNTO RESIDENCIAL NEY BRAGA</t>
         </is>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44">
         <v>0</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>JARDIM IMPERIAL II</t>
+          <t>COPACABANA</t>
         </is>
       </c>
       <c r="B45">
@@ -2385,7 +2487,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>JARDIM INDEPENDENCIA</t>
+          <t>DISTRITO DE FLORIANO FLORIANO</t>
         </is>
       </c>
       <c r="B46">
@@ -2404,26 +2506,26 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>JARDIM INTERNORTE</t>
+          <t>EBENEZER</t>
         </is>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47">
         <v>0</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>JARDIM OASIS</t>
+          <t>IBIRAPUERA</t>
         </is>
       </c>
       <c r="B48">
@@ -2442,7 +2544,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>JARDIM OLIMPICO</t>
+          <t>IGUATEMI</t>
         </is>
       </c>
       <c r="B49">
@@ -2452,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -2461,7 +2563,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>JARDIM OURO COLA</t>
+          <t>JARDIM ALVORADA III</t>
         </is>
       </c>
       <c r="B50">
@@ -2471,7 +2573,7 @@
         <v>0</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -2480,7 +2582,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>JARDIM PINHEIROS III</t>
+          <t>JARDIM ARAUCARIA</t>
         </is>
       </c>
       <c r="B51">
@@ -2499,7 +2601,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>JARDIM SANTA HELENA</t>
+          <t>JARDIM BELA VISTA</t>
         </is>
       </c>
       <c r="B52">
@@ -2509,7 +2611,7 @@
         <v>0</v>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -2518,26 +2620,26 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>JARDIM SANTA ROSA</t>
+          <t>JARDIM BERTIOGA</t>
         </is>
       </c>
       <c r="B53">
         <v>1</v>
       </c>
       <c r="C53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E53">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>JARDIM SAO FRANCISCO</t>
+          <t>JARDIM DIAS I</t>
         </is>
       </c>
       <c r="B54">
@@ -2556,7 +2658,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>JARDIM SAO JORGE</t>
+          <t>JARDIM DO CARMO</t>
         </is>
       </c>
       <c r="B55">
@@ -2575,7 +2677,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>JARDIM SOCIAL</t>
+          <t>JARDIM IMPERIAL II</t>
         </is>
       </c>
       <c r="B56">
@@ -2585,7 +2687,7 @@
         <v>0</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -2594,7 +2696,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>JARDIM UNIVERSO</t>
+          <t>JARDIM INDEPENDENCIA</t>
         </is>
       </c>
       <c r="B57">
@@ -2613,7 +2715,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>JOAO DE BARROS</t>
+          <t>JARDIM INTERNORTE</t>
         </is>
       </c>
       <c r="B58">
@@ -2632,7 +2734,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>KARINA</t>
+          <t>JARDIM IPANEMA</t>
         </is>
       </c>
       <c r="B59">
@@ -2651,7 +2753,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LOT SUMARE</t>
+          <t>JARDIM MARAVILHA</t>
         </is>
       </c>
       <c r="B60">
@@ -2670,7 +2772,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LOTEAMENTO MADRID</t>
+          <t>JARDIM OURO COLA</t>
         </is>
       </c>
       <c r="B61">
@@ -2680,7 +2782,7 @@
         <v>0</v>
       </c>
       <c r="D61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -2689,7 +2791,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MORANGUEIRA</t>
+          <t>JARDIM PAULISTA</t>
         </is>
       </c>
       <c r="B62">
@@ -2708,7 +2810,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NEY BRAGA</t>
+          <t>JARDIM PINHEIROS III</t>
         </is>
       </c>
       <c r="B63">
@@ -2718,7 +2820,7 @@
         <v>0</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -2727,7 +2829,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PARQUE DAS BANDEIRAS</t>
+          <t>JARDIM REAL</t>
         </is>
       </c>
       <c r="B64">
@@ -2746,7 +2848,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PARQUE INDUSTRIAL BANDEIRANTES</t>
+          <t>JARDIM SANTA HELENA</t>
         </is>
       </c>
       <c r="B65">
@@ -2765,26 +2867,26 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PARQUE RESIDENCIAL CIDADE NOVA</t>
+          <t>JARDIM SANTA ROSA</t>
         </is>
       </c>
       <c r="B66">
         <v>1</v>
       </c>
       <c r="C66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PARQUE RESIDENCIAL TUIUTI</t>
+          <t>JARDIM SAO FRANCISCO</t>
         </is>
       </c>
       <c r="B67">
@@ -2803,7 +2905,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PARQUE TARUMA</t>
+          <t>JARDIM SAO JORGE</t>
         </is>
       </c>
       <c r="B68">
@@ -2822,7 +2924,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>PINHEIROS</t>
+          <t>JARDIM SOCIAL</t>
         </is>
       </c>
       <c r="B69">
@@ -2841,7 +2943,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>QUEBEC</t>
+          <t>JARDIM TRES LAGOAS</t>
         </is>
       </c>
       <c r="B70">
@@ -2860,7 +2962,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SAO FRANCISCO</t>
+          <t>JARDIM UNIVERSO</t>
         </is>
       </c>
       <c r="B71">
@@ -2879,7 +2981,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SUMARE</t>
+          <t>JOAO DE BARROS</t>
         </is>
       </c>
       <c r="B72">
@@ -2898,7 +3000,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>TUIUTI</t>
+          <t>KARINA</t>
         </is>
       </c>
       <c r="B73">
@@ -2917,7 +3019,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>VILA ESPERANCA</t>
+          <t>LOT SUMARE</t>
         </is>
       </c>
       <c r="B74">
@@ -2936,7 +3038,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>VILA MARUMBY</t>
+          <t>LOTEAMENTO MADRID</t>
         </is>
       </c>
       <c r="B75">
@@ -2955,7 +3057,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VILA NOVA</t>
+          <t>MORANGUEIRA</t>
         </is>
       </c>
       <c r="B76">
@@ -2974,7 +3076,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VILA SANTA IZABEL</t>
+          <t>NEY BRAGA</t>
         </is>
       </c>
       <c r="B77">
@@ -2984,7 +3086,7 @@
         <v>0</v>
       </c>
       <c r="D77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -2993,7 +3095,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>VILA SANTO ANTONIO</t>
+          <t>PARQUE DAS BANDEIRAS</t>
         </is>
       </c>
       <c r="B78">
@@ -3012,7 +3114,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ZONA 05</t>
+          <t>PARQUE INDUSTRIAL BANDEIRANTES</t>
         </is>
       </c>
       <c r="B79">
@@ -3031,7 +3133,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ZONA 06</t>
+          <t>PARQUE PALMEIRAS</t>
         </is>
       </c>
       <c r="B80">
@@ -3050,7 +3152,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ZONA 08</t>
+          <t>PARQUE RESIDENCIAL CIDADE NOVA</t>
         </is>
       </c>
       <c r="B81">
@@ -3069,7 +3171,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ZONA 3</t>
+          <t>PARQUE RESIDENCIAL TUIUTI</t>
         </is>
       </c>
       <c r="B82">
@@ -3079,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="D82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -3088,19 +3190,247 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>PINHEIROS</t>
+        </is>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>QUEBEC</t>
+        </is>
+      </c>
+      <c r="B84">
+        <v>1</v>
+      </c>
+      <c r="C84">
+        <v>0</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SANTA TEREZINHA</t>
+        </is>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+      <c r="C85">
+        <v>0</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SAO FRANCISCO</t>
+        </is>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+      <c r="C86">
+        <v>0</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SUMARE</t>
+        </is>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TUIUTI</t>
+        </is>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>VILA NOVA</t>
+        </is>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89">
+        <v>0</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>VILA SANTA IZABEL</t>
+        </is>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90">
+        <v>0</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ZONA 05</t>
+        </is>
+      </c>
+      <c r="B91">
+        <v>1</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ZONA 06</t>
+        </is>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92">
+        <v>0</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ZONA 08</t>
+        </is>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ZONA 3</t>
+        </is>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>ZONA 7</t>
         </is>
       </c>
-      <c r="B83">
-        <v>1</v>
-      </c>
-      <c r="C83">
-        <v>0</v>
-      </c>
-      <c r="D83">
-        <v>1</v>
-      </c>
-      <c r="E83">
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95">
+        <v>0</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95">
         <v>0</v>
       </c>
     </row>
@@ -3111,7 +3441,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3144,7 +3474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JARDIM INDEPENDENCIA</t>
+          <t>ALVAMAR</t>
         </is>
       </c>
       <c r="B2">
@@ -3154,7 +3484,7 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -3163,17 +3493,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALVAMAR</t>
+          <t>JARDIM INDEPENDENCIA</t>
         </is>
       </c>
       <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>2</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3182,11 +3512,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JARDIM VERAO</t>
+          <t>PARQUE RESIDENCIAL BOM PASTOR</t>
         </is>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -3201,7 +3531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PARQUE RESIDENCIAL BOM PASTOR</t>
+          <t>COMETA</t>
         </is>
       </c>
       <c r="B5">
@@ -3211,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3220,36 +3550,36 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VERAO</t>
+          <t>INDEPENDENCIA</t>
         </is>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ALPHAVILLE</t>
+          <t>JARDIM VERAO</t>
         </is>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -3258,17 +3588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COMETA</t>
+          <t>PANORAMA</t>
         </is>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -3277,26 +3607,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ESPLANADA</t>
+          <t>VERAO</t>
         </is>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FLORESTA</t>
+          <t>ALPHAVILLE</t>
         </is>
       </c>
       <c r="B10">
@@ -3306,7 +3636,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -3315,7 +3645,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GRALHA AZUL</t>
+          <t>BELA VISTA</t>
         </is>
       </c>
       <c r="B11">
@@ -3334,7 +3664,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA</t>
+          <t>CEREJEIRA</t>
         </is>
       </c>
       <c r="B12">
@@ -3353,7 +3683,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JARDIM NOVA INDEPENDENCIA I</t>
+          <t>ESPLANADA</t>
         </is>
       </c>
       <c r="B13">
@@ -3372,7 +3702,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>JARDIM PANORAMA</t>
+          <t>FLORESTA</t>
         </is>
       </c>
       <c r="B14">
@@ -3391,7 +3721,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JARDIM TRIANGULO</t>
+          <t>GRALHA AZUL</t>
         </is>
       </c>
       <c r="B15">
@@ -3410,7 +3740,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>JARDIM UNIVERSAL</t>
+          <t>JARDIM MONTEREY</t>
         </is>
       </c>
       <c r="B16">
@@ -3429,7 +3759,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MONTEREY</t>
+          <t>JARDIM NOVA INDEPENDENCIA I</t>
         </is>
       </c>
       <c r="B17">
@@ -3448,7 +3778,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NOVA PAULISTA</t>
+          <t>JARDIM PANORAMA</t>
         </is>
       </c>
       <c r="B18">
@@ -3458,7 +3788,7 @@
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -3467,7 +3797,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NOVO PANORAMA</t>
+          <t>JARDIM PERIMETRAL</t>
         </is>
       </c>
       <c r="B19">
@@ -3486,7 +3816,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PARQUE ALVAMAR II</t>
+          <t>JARDIM TRIANGULO</t>
         </is>
       </c>
       <c r="B20">
@@ -3505,19 +3835,133 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>JARDIM UNIVERSAL</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MONTEREY</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NOVA PAULISTA</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NOVO PANORAMA</t>
+        </is>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PARQUE ALVAMAR</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PARQUE ALVAMAR II</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>SAO PAULO</t>
         </is>
       </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
         <v>0</v>
       </c>
     </row>
@@ -3528,7 +3972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3620,7 +4064,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -3640,7 +4084,27 @@
         </is>
       </c>
       <c r="B11">
-        <v>27</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -3650,7 +4114,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3901,7 +4365,7 @@
         </is>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -3923,24 +4387,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SRAG não especificada</t>
+          <t>Outro vírus respiratório</t>
         </is>
       </c>
       <c r="C21">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>SRAG não especificada</t>
         </is>
       </c>
       <c r="C22">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -3949,11 +4413,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C23">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -3962,11 +4426,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Não classificado</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -3975,11 +4439,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Outro vírus respiratório</t>
+          <t>Não classificado</t>
         </is>
       </c>
       <c r="C25">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -3988,24 +4452,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SRAG não especificada</t>
+          <t>Outro vírus respiratório</t>
         </is>
       </c>
       <c r="C26">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>SRAG não especificada</t>
         </is>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -4014,11 +4478,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C28">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -4027,11 +4491,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Não classificado</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -4040,11 +4504,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Outro vírus respiratório</t>
+          <t>Não classificado</t>
         </is>
       </c>
       <c r="C30">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -4053,24 +4517,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SRAG não especificada</t>
+          <t>Outro vírus respiratório</t>
         </is>
       </c>
       <c r="C31">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>SRAG não especificada</t>
         </is>
       </c>
       <c r="C32">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
@@ -4079,7 +4543,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C33">
@@ -4092,11 +4556,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Não classificado</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="C34">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -4105,11 +4569,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Outro vírus respiratório</t>
+          <t>Não classificado</t>
         </is>
       </c>
       <c r="C35">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -4118,24 +4582,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SRAG não especificada</t>
+          <t>Outro vírus respiratório</t>
         </is>
       </c>
       <c r="C36">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>SRAG não especificada</t>
         </is>
       </c>
       <c r="C37">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38">
@@ -4144,11 +4608,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Não classificado</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="C38">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -4157,11 +4621,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Outro vírus respiratório</t>
+          <t>Não classificado</t>
         </is>
       </c>
       <c r="C39">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -4170,7 +4634,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SRAG não especificada</t>
+          <t>Outro vírus respiratório</t>
         </is>
       </c>
       <c r="C40">
@@ -4179,15 +4643,15 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>SRAG não especificada</t>
         </is>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
@@ -4196,11 +4660,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Não classificado</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C42">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -4209,11 +4673,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Outro vírus respiratório</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -4222,11 +4686,128 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>Não classificado</t>
+        </is>
+      </c>
+      <c r="C44">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>10</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Outro vírus respiratório</t>
+        </is>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>10</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>SRAG não especificada</t>
         </is>
       </c>
-      <c r="C44">
-        <v>6</v>
+      <c r="C46">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>11</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Influenza</t>
+        </is>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>11</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Não classificado</t>
+        </is>
+      </c>
+      <c r="C48">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>11</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Outro vírus respiratório</t>
+        </is>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>11</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SRAG não especificada</t>
+        </is>
+      </c>
+      <c r="C50">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>12</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Não classificado</t>
+        </is>
+      </c>
+      <c r="C51">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>12</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Outro vírus respiratório</t>
+        </is>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>12</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SRAG não especificada</t>
+        </is>
+      </c>
+      <c r="C53">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4236,7 +4817,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4358,13 +4939,13 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9">
-        <v>23.1</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="10">
@@ -4375,10 +4956,10 @@
         <v>21</v>
       </c>
       <c r="C10">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="D10">
-        <v>-34.4</v>
+        <v>-32.3</v>
       </c>
     </row>
     <row r="11">
@@ -4386,13 +4967,41 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C11">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D11">
-        <v>28.6</v>
+        <v>76.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>37</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>14</v>
+      </c>
+      <c r="C13">
+        <v>-23</v>
+      </c>
+      <c r="D13">
+        <v>-62.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>